<commit_message>
intergrated with image and search bar
</commit_message>
<xml_diff>
--- a/storage/Prompt Factory.xlsx
+++ b/storage/Prompt Factory.xlsx
@@ -1,18 +1,27 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\142770\Documents\webapp\promptfactory\storage\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0C08091D-D04A-49B7-93A2-E65E949F3E0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <bookViews>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+  </bookViews>
   <sheets>
-    <sheet state="visible" name="PromptDetails" sheetId="1" r:id="rId5"/>
-    <sheet state="visible" name="TeamMembers" sheetId="2" r:id="rId6"/>
+    <sheet name="PromptDetails" sheetId="1" r:id="rId1"/>
+    <sheet name="TeamMembers" sheetId="2" r:id="rId2"/>
   </sheets>
-  <definedNames/>
-  <calcPr/>
+  <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="19" uniqueCount="17">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="36">
   <si>
     <t>PromptID</t>
   </si>
@@ -44,42 +53,9 @@
     <t>https://lokesh-rv.in/prompt/265</t>
   </si>
   <si>
-    <t>Create a high-quality romantic digital watercolor-oil painting portrait of a young South Indian couple, matching the exact face identity, skin tone, hairstyle, facial features, and expressions from the reference photo with zero distortion.
-The woman is standing slightly behind the man, lovingly hugging him from behind with both arms around his shoulders. She is smiling softly, looking down at him with affection. She has expressive eyes, a small red bindi, subtle natural makeup, traditional gold jhumka earrings, and neatly styled hair with soft loose strands. She is wearing a green saree with an elegant, soft fabric texture..
-The man is smiling warmly and looking up at the woman with affection. He has voluminous styled dark hair, light stubble beard, and is wearing a casual red shirt.
-Art style should be a realistic hand-painted watercolor and oil painting blend, with visible brush strokes, rich texture, smooth natural skin tones, and soft edges.
-Use warm natural lighting, pastel background)</t>
-  </si>
-  <si>
-    <t>Couple</t>
-  </si>
-  <si>
     <t xml:space="preserve">Gpt </t>
   </si>
   <si>
-    <t>Edit a realistic portrait from the original reference image with 10000% exact facial likeness, with no changes to the face at all.
-Ultra photorealistic lifestyle photography, natural candid couple moment, cinematic realism, high detail, soft sunlight. 3-frame vertical collage composition telling a sequence of moments.
-Scene set in a lush outdoor flower shop, filled with colorful flower pots, green plants, and fresh blossoms arranged densely but naturally. Midday sunlight lights the scene with natural daylight, soft shadows, bright yet realistic colors.
-The subjects are a young man and woman with warm chemistry and happy expressions.
-Woman: Wearing a sleeveless white dress with a loose, flowy cut, lightweight fabric moving in the wind, feminine and romantic style. Short black hair styled naturally, decorated with a red flower on the side of the hair, cheerful expression, open smile, playful and loving body language.
-Man: Wearing a loose light blue shirt and white pants, clean and casual style. Neatly natural black hair, relaxed and warm expression. Holding a fresh bouquet of flowers in pink and pastel colors.
-Scene frames: – Standing side by side in front of the flower shop, relaxed and playful pose. – A close interaction moment as the man gives her the bouquet, spontaneous laughter, eye contact full of emotion. – A cute and intimate pose with their bodies leaning against each other, showing closeness and happiness.
-Overall visual style: romantic slice of life, Japanese / Korean indie film aesthetic, documentary photography feel, candid emotion, no-pose look, natural imperfection, realistic skin texture, slightly shallow depth of field, true-to-life color grading, nostalgic yet fresh mood.
-Vertical aspect ratio, balanced composition, sharp plant details, a warm and lively spring / summer romance atmosphere.
-⚙️ MIDJOURNEY v6 – RECOMMENDED PARAMETERS
-Add this at the end of the prompt:
---v 6 --style raw --ar 4:5 --chaos 6 --quality 1 
-⚙️ SDXL – PHOTOREAL PRESET (RECOMMENDED)
-Sampler: DPM++ 2M Karras
-Steps: 30–40
-CFG Scale: 4 – 6
-Resolution: 1024×1280 / 1536×1920
-Hires Fix / Refiner: ON
-Refiner Strength: 0.2 – 0.3
-🚫 NEGATIVE PROMPT (IMPORTANT)
-low resolution, low quality, blurry, motion blur, pixelated, noise, grainy, overexposed, underexposed, harsh lighting, studio lighting, artificial light, beauty filter, over-smooth skin, plastic skin, doll face, anime, cartoon, illustration, painting, CGI, 3D render, distorted anatomy, extra limbs, extra fingers, bad hands, stiff pose, forced pose, fake emotion, awkward interaction, oversaturated colors, heavy color grading, HDR look, watermark, logo, text, UI elements, frame, cropped head, cropped body --v 6 --style raw --ar 4:5 --chaos 6 --quality 1</t>
-  </si>
-  <si>
     <t>Kathir</t>
   </si>
   <si>
@@ -87,27 +63,177 @@
   </si>
   <si>
     <t>Baskaran</t>
+  </si>
+  <si>
+    <t>Use the uploaded reference image as the single and absolute source of identity. Reproduce the same young adult South Asian woman with 100% facial accuracy, preserving exact face shape, bone structure, jawline, cheekbones, nose size and length, lip shape, eye shape, eyelids, eyebrow thickness, forehead height, skin texture, and natural asymmetry exactly as in the uploaded image. Do not beautify, idealize, stylize facial proportions, change age, ethnicity, expression, or identity. The face must remain unmistakably the same person, with realism translated faithfully into illustration form.
+Render the subject as a vintage-style illustration with gritty, distressed, old print texture, resembling hand screen-printed posters or old comic art, with visible grain, ink noise, slight misregistration, and worn paper feel, while maintaining strict facial likeness.
+The woman stands in the aisle of an old public bus, viewed from a low-angle perspective looking toward the front. She wears a traditional Indian sari draped in a simple, functional everyday style, deep warm brown with a subtle sheen, paired with a dark short-sleeved blouse. Lighting dramatically highlights her face and the folds of the sari, creating a stark, cinematic mood.
+The bus interior is heavily stylized with Indian folk-art hand-painted details, dominated by teal, dark green, earthy brown, and muted yellow-gold tones. The ceiling is teal with geometric and floral patterns in faded gold and yellow. Upper window panels are teal with intricate decorative painting. Seats on both sides of the aisle are dark green with worn brown cushions showing age and use.
+Strong diffused daylight enters through the front windshield, resembling early sunrise or harsh morning light, filtered through striped hanging cloths or banners in orange, yellow, and blue. On the right near the front, a white rectangular box with red text reading exactly “FIRST AID BOX” is visible, and below it a large stylized painted deity-like eye in yellow, green, and black. Further back above the windows, small aged framed devotional images are present.
+The overall aesthetic is dramatic, cinematic, grounded, and authentic, with no modern elements, no clean surfaces, and no digital polish. Vertical poster-style composition, centered subject, strong leading lines from bus seats, face clearly readable. No face swap, no generic AI face, no beauty filters, no smooth plastic skin, no anime, no cartoon, no Pixar or Disney style, no incorrect text, no altered signage, no modern bus interiors. If any conflict arises between style and likeness, likeness must always win.</t>
+  </si>
+  <si>
+    <t>Women</t>
+  </si>
+  <si>
+    <t>Women,portrait</t>
+  </si>
+  <si>
+    <t>Women,portrait,indian-culture</t>
+  </si>
+  <si>
+    <t>A photorealistic, high-angle snapshot of a young Indian woman sitting on the floor indoors. She has long straight dark hair with a middle part and a small red bindi on her forehead.She is wearing a bright orange shortsleeved blouse with gold embroidery and green borders, paired with a dark kanjivaram brown saree. She is wearing stacks of dark maroon and sparkling silver bangles on her wrists. For makeup natural glam makeup glossy nude-pink lips, nude-pink dewy blushShe is posing coyly, leaning
+forward slightly, with the back of her left handgently touching her chin, looking into camera to the side. Background features a plain white wall, a small wooden stool with bright pink orchids to her left, and a potted red rose plant to her right. The floor has a grey and white striped rug. Lighting is harsh, direct on-camera flash photography style, creating hard shadows behind the plants, vintage 2000s aesthetic, candid vibe, sharp focus on the face no facial change same as it is on the
+picture.. Create this referance image image id and face shuld not be changed at all. 9:16 girl eye open
+Create this referance image image id and face shuld not be changed at all.". copy my face 100% dont change the face. Create this referance image image id and face shuld not be changed at all. 3:4retio image</t>
+  </si>
+  <si>
+    <t>Buat saya memakai kostum qin shi huang dari anime record of ragnarok, termasuk desain penutup mata dan pakaian yang di kenakan qin shi huang di dalam anime record of ragnarok. Buatkan pose khas nya
+characterized by stark cinematic lighting and intense contrast. Captured with a slightly low, upward-facing angle that dramatizes the subject's jawline and neck, the composition evokes quiet dominance and sculptural elegance. The background is a deep, saturated crimson red, creating a bold visual clash with the model's luminous skin and dark wardrobe. Lighting is tightly directional, casting warm golden highlights on one side of the face while plunging the other into velvety shadow, emphasizing bone structure with almost architectural
+precision.
+The subject's expression is unreadable and
+cool-toned-eyes half-lidded, lips relaxed- suggesting detachment or quiet defiance. The model wears a heavy wool or felt overcoat, its texture richly defined against the skin's smooth, dewy glow. Minimal retouching preserves skin texture and slight imperfections, adding realism. Editorial tension is created through close cropping, tonal control, and the almost oppressive intimacy of the camera's proximity. There are no props or accessories; the visual impact is created purely through light, shadow, color saturation, and posture - evoking high fashion, contemporary isolation, and hyper-modern masculinity. Make the face and hairstyle as similar as possible to the one in the photo. Buat kostumnya sangat detail dan realistis.
+Pertahankan gaya rambut dan warna yang sama, Gunakan warna dan tekstur yang mirip anime.</t>
+  </si>
+  <si>
+    <t>Men</t>
+  </si>
+  <si>
+    <t>Men,portrait</t>
+  </si>
+  <si>
+    <t>Transform the uploaded real person into a soft comic illustration.
+Important rules:
+Keep the face exactly the same
+Do not change facial features or expressions
+Do not beautify or stylize the face
+Keep the outfit exactly the same as the original image
+Panels:
+Casual top-down candid shot, sitting naturally and holding a phone
+Close-up of the eyes with soft reflections
+Main scene showing a natural smile or laugh, head slightly tilted, relaxed posture
+Details:
+Gentle natural blush
+Visible skin texture and tiny smile lines
+Loose hair strands, hairstyle unchanged
+Art style:
+Clean anime-style linework
+Soft matte digital coloring
+Simple cel shading
+Light paper-like texture
+Background &amp; details:
+Hand-drawn sparkle icons
+Soft linen paper texture overlay
+Minimal cute doodles, very subtle
+Colors:
+Original outfit colors
+Soft pastel background tones
+Lighting:
+Soft natural daylight, even and gentle
+Overall look:
+Cozy, nostalgic, comic illustration.</t>
+  </si>
+  <si>
+    <t>Women,cartoon</t>
+  </si>
+  <si>
+    <t>A slim, elegant 5'7 young woman riding a powerful black hairy horse, captured from a frontside angle (three-quarter frontal view). The camera is positioned slightly lower, facing her as the horse moves forward, creating a bold, confident, cinematic presence. She glances subtly to the side with a calm, fearless expression, her full face clearly visible.
+She sits upright and perfectly balanced, holding the reins naturally while leaning slightly into the horse’s forward motion, conveying control, grace, and strength. The horse appears muscular and majestic, with a thick flowing mane, captured mid-stride to emphasize raw power, speed, and motion.
+She wears an oversized white linen shirt with the top buttons softly open, styled effortlessly over light blue baggy jeans. Clean white Nike Air Force 1 sneakers ground the look with modern street elegance. A delicate silver wristwatch catches light on her wrist, while narrow-frame rectangular classy sunglasses enhance her confident, contemporary aesthetic.
+Her face must be preserved 100% exactly as provided from the reference image. Do NOT alter facial structure, proportions, skin texture, eye shape, nose, lips, jawline, expression, or identity. No beautification, no face swap, no smoothing, no AI modification of facial features.
+The background is heavily motion-blurred with directional streaks clearly indicating forward movement, while the woman and horse remain sharp and in perfect focus. Dust particles and subtle motion blur around the horse’s legs add realism and cinematic speed.
+The image features a vintage cinematic grain aesthetic inspired by Leica M11 Monochrome, with rich black-and-white tones, deep contrast, dramatic shadows, soft highlights, and a timeless editorial mood. Subtle film grain and cinematic depth of field enhance the high-end fashion photography feel.
+Ultra-realistic, cinematic composition, shallow depth of field, dynamic motion blur, dramatic storytelling, monochrome masterpiece.</t>
+  </si>
+  <si>
+    <t>A slim-fit 5'7 young man riding a powerful black hairy horse, captured from a frontside angle (three-quarter frontal view). The camera is positioned slightly lower, facing him as the horse moves forward, creating a strong, confident cinematic presence. He is glancing slightly to the side with a composed, fearless expression, fully visible face.
+He sits upright and balanced, holding the reins naturally while leaning subtly into the horse's forward motion. The horse is muscular and majestic, with a thick flowing mane, captured mid-stride, emphasizing strength and speed.
+He is wearing an oversized white linen shirt with the top buttons open, light blue baggy jeans, and clean white Nike Air Force 1 sneakers. A subtle silver wristwatch reflects light on his wrist, and narrow-frame rectangular classy sunglasses complete his modern, stylish look.
+His face must be preserved 100% exactly as provided. Do NOT change facial structure, proportions, skin texture, eye shape, nose, lips, jawline, expression, or identity. No beautification, no face swap, no smoothing, no Al alteration of facial features.
+The background is strongly motion-blurred, with streaking blur lines to clearly indicate forward movement, while the subject and horse remain sharp and in focus. Dust particles and slight blur around the horse's legs enhance realism and dynamic speed.
+The image features a vintage cinematic grain aesthetic, inspired by Leica M11
+Monochrome, with rich black-and-white tones, deep contrast, dramatic shadows, soft highlights, and a timeless editorial feel. Add subtle film grain and cinematic depth of field for a high-end fashion photography look.
+Ultra-realistic, cinematic composition, shallow depth of field, dynamic motion blur, dramatic storytelling, monochrome masterpiece.</t>
+  </si>
+  <si>
+    <t>Women,Sports</t>
+  </si>
+  <si>
+    <t>Men,Sports</t>
+  </si>
+  <si>
+    <t>{
+"prompt": "Ultra-realistic 8K photograph, 9:16 vertical. Preserve my face 100% exactly as the uploaded reference image (no facial modification, no beautification, no identity change). A young woman standing and lightly leaning near the hood of a black BMW M5 Competition, matching the exact reference pose, body posture, hand placement, facial expression, and camera angle. She is slightly looking left beside the car on a mountain road. She wears wraparound Y2K sunglasses and a cute sporty costume suit inspired by motorsport street fashion: a black cropped oversized hoodie-style top with a small BMW logo on the right chest, a small M-series logo on the left chest, and the word 'MOTORSPORTS' printed vertically down the center. She wears high-waist baggy grey-black cargo pants and clean white Air Force–style sneakers. She lightly holds a Red Bull can in her right hand while her left hand rests on her stomach. The BMW M5 Competition must remain identical with black metallic paint, aggressive front grille, accurate reflections, and Indian license plate 'HR 01 A 0001'. Background replaced with hyper-realistic Meghalaya scenery: lush green rolling hills, misty layered mountains, tall scattered pine trees, soft clouds, clean air, and natural greenery. Road blends naturally into the Meghalaya landscape. No blur anywhere; everything must be sharp and realistic. Lighting matches an overcast Meghalaya morning with soft diffused daylight, realistic shadows, reflections, and weather coherence.",
+"camera": {
+"type": "iPhone 17 Pro Max",
+"lens": "Main 1× Lens",
+"aperture": "f/1.5",
+"shutter_speed": "1/180",
+"iso": "50",
+"white_balance": "cool overcast daylight",
+"focus": "sharp on subject and background"
+},
+"enhance": {
+"skin": "natural texture, realistic pores, no smoothing",
+"lighting": "soft diffused Meghalaya daylight",
+"details": "sharp fabric texture, crisp car reflections, highly detailed Meghalaya hills and greenery, no blur anywhere"
+},
+"negative_prompt": "no blur, no pose change, no body angle change, no facial alteration, no outfit change, no car change, no different scenery except Meghalaya, no CGI look, no extra people, no extra objects, no distortion, no low realism"
+}</t>
+  </si>
+  <si>
+    <t>Men,Outdoor,Car</t>
+  </si>
+  <si>
+    <t>A photograph captures a woman, She is wearing a traditional Indian saree in a deep, vibrant red and orange color, draped elegantly. Her hair is pulled back in a neat bun, adorned with a gold-colored maang tikka on her forehead and white flowers (gajra) woven into the bun. She has several pieces of gold-colored jewelry, including large chandelier earrings, a necklace with a pendant, and multiple bangles on both wrists. She has a dark bindi on her forehead and her smile suggests contentment or engagement in the activity.
+The woman is positioned slightly to the right of the center, kneeling on a paved or tiled outdoor surface. She is pouring a liquid from a small, shiny silver plate or tray into a dark brown clay pot (kalash or matka), which is resting on a smaller, similar-colored clay stand or stove (chulha). The pot is decorated with green leaves and what appear to be turmeric rhizomes or similar stalks tied to its neck. She holds the plate with both hands, tilting it carefully.
+In the background, there is a dense, tall hedge or row of dark green foliage, suggesting a garden or outdoor setting. The lighting is bright and natural, indicating daylight, and there is a soft focus on the background, bringing the subject and the ritual objects into sharp focus. The paved ground beneath the pot and the woman is made of light-colored, possibly grey, square or rectangular tiles or stone.
+The image is taken at a medium close-up level, focusing intently on the ritual activity.</t>
+  </si>
+  <si>
+    <t>Women,traditional</t>
+  </si>
+  <si>
+    <t>Women,traditional,Pongal</t>
+  </si>
+  <si>
+    <t>A portrait-oriented image captures a young woman standing beside a black ox in a rural, outdoor setting, likely a rice paddy or field, with palm trees in the background. The woman appears to be in her 20s South Asian ethnicity, possibly Indian, given her attire. She is smiling and gently touching the ox's face with her right hand.
+She is dressed in traditional South Asian attire, specifically a bright magenta or hot pink silk saree with a gold border, draped over a purple blouse embroidered with gold thread. Her jewelry includes a gold necklace, matching gold dangling earrings, and gold bangles on her wrist. She also has a small black bindi or mark between her eyebrows.
+The ox is a large, dark black or dark brown animal with impressive, curved horns. Its head and horns are elaborately decorated for a festive occasion. A garland of bright red flowers encircles its head, and a yellow ribbon is tied between its horns, adorned with red and yellow pom-poms on the tips. A long garland made of white and green flowers, interspersed with red accents, hangs down its face and neck. A red and yellow braided rope is used as a bridle, tied around its snout and neck.
+To the left of the woman, partially visible, is the arm and torso of another individual, inferred to be a man, wearing a rustic red shirt. His skin tone is dark brown, and he is holding a thick length of brown rope, likely associated with the ox.
+The background consists of a lush green field, possibly a rice field, stretching into the distance. A line of tall palm trees forms a dense backdrop under an overcast or pale sky, suggesting a natural, agricultural environment. The lighting is soft and diffused, typical of an overcast day.</t>
+  </si>
+  <si>
+    <t>a man standing next to a decorated bull against a dark, purple-hued background. The man appears to be an adult He is wearing traditional South Indian attire consisting of a white dhoti wrapped around his waist and legs, and a red shirt worn open over a white undershirt or vest. The red shirt is unbuttoned at the top, revealing a thin chain or pendant. The man is standing with his weight shifted to his left leg, his right arm resting on the bull's back, and his left hand placed on his hip. He is looking directly at the viewer with a slight smile.
+To his right is a large bull with dark brown and white coloring, particularly around the face and body. The bull has long, cream-colored horns that curve slightly upwards. The bull's head and neck are heavily decorated with garlands of pink and red flowers, and a white flower arrangement is placed between its horns. A thick rope or bridle, also decorated with flowers, is around its muzzle. The bull is facing the viewer, slightly angled towards the man.
+The background is a dark blur</t>
+  </si>
+  <si>
+    <t>Men,traditional,Pongal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-  <fonts count="3">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <sz val="10.0"/>
+      <sz val="10"/>
       <color rgb="FF000000"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="10"/>
       <color theme="1"/>
       <name val="Arial"/>
       <scheme val="minor"/>
     </font>
     <font>
       <u/>
+      <sz val="10"/>
       <color rgb="FF0000FF"/>
+      <name val="Arial"/>
     </font>
   </fonts>
   <fills count="2">
@@ -115,47 +241,50 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="lightGray"/>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" applyAlignment="1" applyFont="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
-    <xf borderId="0" fillId="0" fontId="0" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0" shrinkToFit="0" vertical="bottom" wrapText="0"/>
+  <cellXfs count="5">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
-    </xf>
-    <xf borderId="0" fillId="0" fontId="2" numFmtId="0" xfId="0" applyAlignment="1" applyFont="1">
-      <alignment readingOrder="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle xfId="0" name="Normal" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+    <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{9260A510-F301-46a8-8635-F512D64BE5F5}">
+      <x15:timelineStyles defaultTimelineStyle="TimeSlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
 </file>
 
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<x18tc:personList xmlns:x18tc="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments"/>
-</file>
-
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheets">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Sheets">
   <a:themeElements>
     <a:clrScheme name="Sheets">
       <a:dk1>
@@ -345,21 +474,25 @@
       </a:bgFillStyleLst>
     </a:fmtScheme>
   </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
 </a:theme>
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="A1:I11"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col customWidth="1" min="6" max="6" width="13.88"/>
-    <col customWidth="1" min="7" max="7" width="12.5"/>
+    <col min="5" max="5" width="24.453125" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="13.90625" customWidth="1"/>
+    <col min="7" max="7" width="12.453125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -388,68 +521,166 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2">
+    <row r="2" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
-        <v>1.0</v>
+        <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="I2" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="D2" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I2" s="1" t="s">
-        <v>12</v>
-      </c>
-    </row>
-    <row r="3">
+    </row>
+    <row r="3" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
-        <v>2.0</v>
-      </c>
-      <c r="C3" s="1" t="s">
-        <v>13</v>
+        <v>2</v>
+      </c>
+      <c r="C3" s="3" t="s">
+        <v>18</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>11</v>
+        <v>15</v>
+      </c>
+      <c r="E3" t="s">
+        <v>16</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E4" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C5" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E5" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C6" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E6" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C7" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E7" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C8" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E8" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C9" s="4" t="s">
+        <v>30</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E9" t="s">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C10" s="4" t="s">
+        <v>33</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="E10" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C11" s="4" t="s">
+        <v>34</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E11" t="s">
+        <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink r:id="rId1" ref="B2"/>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
   </hyperlinks>
-  <drawing r:id="rId2"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <dimension ref="B2:B4"/>
+  <sheetFormatPr defaultColWidth="12.6328125" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="2">
+    <row r="2" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B2" s="1" t="s">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="3">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B3" s="1" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="4">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="B4" s="1" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
     </row>
   </sheetData>
-  <drawing r:id="rId1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>